<commit_message>
clean version of thread summary
</commit_message>
<xml_diff>
--- a/thread-strength/03_analyses/assemble-thread-summary/thread-summary-gallo.xlsx
+++ b/thread-strength/03_analyses/assemble-thread-summary/thread-summary-gallo.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="184">
   <si>
     <t xml:space="preserve">sort_ID</t>
   </si>
@@ -143,10 +143,10 @@
     <t xml:space="preserve">G017_4</t>
   </si>
   <si>
-    <t xml:space="preserve">G18_1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G18</t>
+    <t xml:space="preserve">G018_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G018</t>
   </si>
   <si>
     <t xml:space="preserve">control</t>
@@ -158,19 +158,13 @@
     <t xml:space="preserve">try2</t>
   </si>
   <si>
-    <t xml:space="preserve">G018_1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G018</t>
-  </si>
-  <si>
     <t xml:space="preserve">thread broke at .235 N. broke again at .31 N. broke again at .375 N</t>
   </si>
   <si>
     <t xml:space="preserve">tryTwo</t>
   </si>
   <si>
-    <t xml:space="preserve">G18_2</t>
+    <t xml:space="preserve">G018_2</t>
   </si>
   <si>
     <t xml:space="preserve">G018_3</t>
@@ -179,37 +173,37 @@
     <t xml:space="preserve">thread broke at .23 N. grabbed remainder and retested, broke again at .34 N</t>
   </si>
   <si>
-    <t xml:space="preserve">G19_1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G19</t>
+    <t xml:space="preserve">G019_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G019</t>
   </si>
   <si>
     <t xml:space="preserve">thread at 0.175 N</t>
   </si>
   <si>
-    <t xml:space="preserve">G19_2</t>
+    <t xml:space="preserve">G019_2</t>
   </si>
   <si>
     <t xml:space="preserve">thread at 0.465 N</t>
   </si>
   <si>
-    <t xml:space="preserve">G19_3</t>
+    <t xml:space="preserve">G019_3</t>
   </si>
   <si>
     <t xml:space="preserve">thread at 0.085. restested: thread again at 0.265</t>
   </si>
   <si>
-    <t xml:space="preserve">G19_4</t>
+    <t xml:space="preserve">G019_4</t>
   </si>
   <si>
     <t xml:space="preserve">thread at 0.505 N</t>
   </si>
   <si>
-    <t xml:space="preserve">G20_1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G20</t>
+    <t xml:space="preserve">G020_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G020</t>
   </si>
   <si>
     <t xml:space="preserve">OW</t>
@@ -218,12 +212,6 @@
     <t xml:space="preserve">tearing</t>
   </si>
   <si>
-    <t xml:space="preserve">G020_1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G020</t>
-  </si>
-  <si>
     <t xml:space="preserve">thread broke at .105 N. got reimainder of thread and tested again</t>
   </si>
   <si>
@@ -236,13 +224,13 @@
     <t xml:space="preserve">was already coming off by the time i started the force test</t>
   </si>
   <si>
-    <t xml:space="preserve">G20_4</t>
+    <t xml:space="preserve">G020_4</t>
   </si>
   <si>
     <t xml:space="preserve">thread at .225 N</t>
   </si>
   <si>
-    <t xml:space="preserve">G20_5</t>
+    <t xml:space="preserve">G020_5</t>
   </si>
   <si>
     <t xml:space="preserve">G021_1</t>
@@ -254,67 +242,58 @@
     <t xml:space="preserve">G021_2</t>
   </si>
   <si>
-    <t xml:space="preserve">G22_2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G22</t>
+    <t xml:space="preserve">G022_2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G022</t>
   </si>
   <si>
     <t xml:space="preserve">thread at 0.05</t>
   </si>
   <si>
-    <t xml:space="preserve">G22_3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G23_1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G23_3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G23_4</t>
+    <t xml:space="preserve">G022_3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G023_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G023_3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G023_4</t>
   </si>
   <si>
     <t xml:space="preserve">thread at 0.095</t>
   </si>
   <si>
-    <t xml:space="preserve">G24_1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G24</t>
-  </si>
-  <si>
     <t xml:space="preserve">G024_1</t>
   </si>
   <si>
     <t xml:space="preserve">G024</t>
   </si>
   <si>
-    <t xml:space="preserve">G24_2</t>
-  </si>
-  <si>
     <t xml:space="preserve">G024_2</t>
   </si>
   <si>
-    <t xml:space="preserve">G24_3</t>
+    <t xml:space="preserve">G024_3</t>
   </si>
   <si>
     <t xml:space="preserve">G024_4</t>
   </si>
   <si>
-    <t xml:space="preserve">G25_1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G25_2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G25_3</t>
+    <t xml:space="preserve">G025_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G025_2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G025_3</t>
   </si>
   <si>
     <t xml:space="preserve">G026_1</t>
@@ -338,46 +317,46 @@
     <t xml:space="preserve">thread broke at .185 N</t>
   </si>
   <si>
-    <t xml:space="preserve">G28_1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G28</t>
+    <t xml:space="preserve">G028_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G028</t>
   </si>
   <si>
     <t xml:space="preserve">DO</t>
   </si>
   <si>
-    <t xml:space="preserve">G30_1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G30_2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G30_3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G31_1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G31</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G31_2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G32_1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G32</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G32_2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G32_3</t>
+    <t xml:space="preserve">G030_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G030</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G030_2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G030_3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G031_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G031</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G031_2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G032_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G032</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G032_2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G032_3</t>
   </si>
   <si>
     <t xml:space="preserve">G071_1</t>
@@ -1717,10 +1696,10 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="B17" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C17" t="n">
         <v>1</v>
@@ -1756,7 +1735,7 @@
       <c r="N17"/>
       <c r="O17"/>
       <c r="P17" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="Q17" t="s">
         <v>23</v>
@@ -1764,10 +1743,10 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="B18" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C18" t="n">
         <v>1</v>
@@ -1803,7 +1782,7 @@
       <c r="N18"/>
       <c r="O18"/>
       <c r="P18" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="Q18" t="s">
         <v>23</v>
@@ -1811,16 +1790,16 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="B19" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C19" t="n">
         <v>1</v>
       </c>
       <c r="D19" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E19" t="s">
         <v>6</v>
@@ -1850,7 +1829,7 @@
       <c r="N19"/>
       <c r="O19"/>
       <c r="P19" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="Q19" t="s">
         <v>23</v>
@@ -1858,7 +1837,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B20" t="s">
         <v>44</v>
@@ -1909,10 +1888,10 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B21" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C21" t="n">
         <v>3</v>
@@ -1948,7 +1927,7 @@
       <c r="N21"/>
       <c r="O21"/>
       <c r="P21" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="Q21" t="s">
         <v>23</v>
@@ -1956,16 +1935,16 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B22" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C22" t="n">
         <v>3</v>
       </c>
       <c r="D22" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E22" t="s">
         <v>6</v>
@@ -1995,7 +1974,7 @@
       <c r="N22"/>
       <c r="O22"/>
       <c r="P22" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="Q22" t="s">
         <v>23</v>
@@ -2003,10 +1982,10 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C23" t="n">
         <v>1</v>
@@ -2042,7 +2021,7 @@
       <c r="N23"/>
       <c r="O23"/>
       <c r="P23" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="Q23" t="s">
         <v>23</v>
@@ -2050,10 +2029,10 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B24" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C24" t="n">
         <v>2</v>
@@ -2089,7 +2068,7 @@
       <c r="N24"/>
       <c r="O24"/>
       <c r="P24" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="Q24" t="s">
         <v>23</v>
@@ -2097,10 +2076,10 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B25" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C25" t="n">
         <v>3</v>
@@ -2136,7 +2115,7 @@
       <c r="N25"/>
       <c r="O25"/>
       <c r="P25" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="Q25" t="s">
         <v>23</v>
@@ -2144,10 +2123,10 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B26" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C26" t="n">
         <v>3</v>
@@ -2183,7 +2162,7 @@
       <c r="N26"/>
       <c r="O26"/>
       <c r="P26" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="Q26" t="s">
         <v>23</v>
@@ -2191,10 +2170,10 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B27" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C27" t="n">
         <v>4</v>
@@ -2230,7 +2209,7 @@
       <c r="N27"/>
       <c r="O27"/>
       <c r="P27" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="Q27" t="s">
         <v>23</v>
@@ -2238,10 +2217,10 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B28" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C28" t="n">
         <v>1</v>
@@ -2259,7 +2238,7 @@
         <v>45</v>
       </c>
       <c r="H28" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I28" t="n">
         <v>0.105</v>
@@ -2274,7 +2253,7 @@
         <v>34.4262295081967</v>
       </c>
       <c r="M28" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="N28" t="n">
         <v>0.105</v>
@@ -2289,10 +2268,10 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="B29" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C29" t="n">
         <v>1</v>
@@ -2307,10 +2286,10 @@
         <v>20</v>
       </c>
       <c r="G29" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H29" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I29" t="n">
         <v>0.22</v>
@@ -2334,7 +2313,7 @@
         <v>0</v>
       </c>
       <c r="P29" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="Q29" t="s">
         <v>23</v>
@@ -2342,10 +2321,10 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="B30" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C30" t="n">
         <v>1</v>
@@ -2360,10 +2339,10 @@
         <v>20</v>
       </c>
       <c r="G30" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H30" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I30" t="n">
         <v>0.105</v>
@@ -2387,7 +2366,7 @@
         <v>-0.115</v>
       </c>
       <c r="P30" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="Q30" t="s">
         <v>23</v>
@@ -2395,10 +2374,10 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B31" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C31" t="n">
         <v>2</v>
@@ -2413,10 +2392,10 @@
         <v>20</v>
       </c>
       <c r="G31" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H31" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I31" t="n">
         <v>0.13</v>
@@ -2446,10 +2425,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B32" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C32" t="n">
         <v>3</v>
@@ -2464,10 +2443,10 @@
         <v>20</v>
       </c>
       <c r="G32" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H32" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I32" t="n">
         <v>0.04</v>
@@ -2491,7 +2470,7 @@
         <v>0</v>
       </c>
       <c r="P32" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="Q32" t="s">
         <v>23</v>
@@ -2499,10 +2478,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B33" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C33" t="n">
         <v>4</v>
@@ -2520,7 +2499,7 @@
         <v>45</v>
       </c>
       <c r="H33" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I33" t="n">
         <v>0.225</v>
@@ -2538,7 +2517,7 @@
       <c r="N33"/>
       <c r="O33"/>
       <c r="P33" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="Q33" t="s">
         <v>23</v>
@@ -2546,10 +2525,10 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B34" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C34" t="n">
         <v>5</v>
@@ -2567,7 +2546,7 @@
         <v>45</v>
       </c>
       <c r="H34" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I34" t="n">
         <v>0.175</v>
@@ -2597,10 +2576,10 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B35" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C35" t="n">
         <v>1</v>
@@ -2615,10 +2594,10 @@
         <v>20</v>
       </c>
       <c r="G35" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H35" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I35" t="n">
         <v>0.18</v>
@@ -2648,10 +2627,10 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B36" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C36" t="n">
         <v>2</v>
@@ -2666,10 +2645,10 @@
         <v>20</v>
       </c>
       <c r="G36" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H36" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I36" t="n">
         <v>0.215</v>
@@ -2684,7 +2663,7 @@
         <v>64.5645645645646</v>
       </c>
       <c r="M36" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="N36" t="n">
         <v>0.215</v>
@@ -2699,10 +2678,10 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B37" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C37" t="n">
         <v>2</v>
@@ -2720,7 +2699,7 @@
         <v>45</v>
       </c>
       <c r="H37" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I37" t="n">
         <v>0.05</v>
@@ -2738,7 +2717,7 @@
       <c r="N37"/>
       <c r="O37"/>
       <c r="P37" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="Q37" t="s">
         <v>23</v>
@@ -2746,10 +2725,10 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B38" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C38" t="n">
         <v>3</v>
@@ -2767,7 +2746,7 @@
         <v>45</v>
       </c>
       <c r="H38" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I38" t="n">
         <v>0.065</v>
@@ -2797,10 +2776,10 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B39" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C39" t="n">
         <v>1</v>
@@ -2818,7 +2797,7 @@
         <v>45</v>
       </c>
       <c r="H39" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I39" t="n">
         <v>0.15</v>
@@ -2848,10 +2827,10 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B40" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C40" t="n">
         <v>3</v>
@@ -2869,7 +2848,7 @@
         <v>45</v>
       </c>
       <c r="H40" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I40" t="n">
         <v>0.02</v>
@@ -2899,10 +2878,10 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B41" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C41" t="n">
         <v>4</v>
@@ -2920,7 +2899,7 @@
         <v>45</v>
       </c>
       <c r="H41" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I41" t="n">
         <v>0.095</v>
@@ -2938,7 +2917,7 @@
       <c r="N41"/>
       <c r="O41"/>
       <c r="P41" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="Q41" t="s">
         <v>23</v>
@@ -2946,10 +2925,10 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B42" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C42" t="n">
         <v>1</v>
@@ -2967,7 +2946,7 @@
         <v>45</v>
       </c>
       <c r="H42" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I42" t="n">
         <v>0.115</v>
@@ -2997,10 +2976,10 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="B43" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="C43" t="n">
         <v>1</v>
@@ -3015,10 +2994,10 @@
         <v>20</v>
       </c>
       <c r="G43" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H43" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I43" t="n">
         <v>0.11</v>
@@ -3048,10 +3027,10 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="B44" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C44" t="n">
         <v>2</v>
@@ -3069,7 +3048,7 @@
         <v>45</v>
       </c>
       <c r="H44" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I44" t="n">
         <v>0.18</v>
@@ -3099,10 +3078,10 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="B45" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="C45" t="n">
         <v>2</v>
@@ -3117,10 +3096,10 @@
         <v>20</v>
       </c>
       <c r="G45" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H45" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I45" t="n">
         <v>0.15</v>
@@ -3150,10 +3129,10 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="B46" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C46" t="n">
         <v>3</v>
@@ -3171,7 +3150,7 @@
         <v>45</v>
       </c>
       <c r="H46" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I46" t="n">
         <v>0.025</v>
@@ -3201,10 +3180,10 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="B47" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="C47" t="n">
         <v>4</v>
@@ -3219,10 +3198,10 @@
         <v>20</v>
       </c>
       <c r="G47" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H47" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I47" t="n">
         <v>0.095</v>
@@ -3252,10 +3231,10 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="B48" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="C48" t="n">
         <v>1</v>
@@ -3273,7 +3252,7 @@
         <v>45</v>
       </c>
       <c r="H48" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I48" t="n">
         <v>0.13</v>
@@ -3303,10 +3282,10 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="B49" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="C49" t="n">
         <v>2</v>
@@ -3324,7 +3303,7 @@
         <v>45</v>
       </c>
       <c r="H49" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I49" t="n">
         <v>0.29</v>
@@ -3354,10 +3333,10 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="B50" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="C50" t="n">
         <v>3</v>
@@ -3375,7 +3354,7 @@
         <v>45</v>
       </c>
       <c r="H50" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I50" t="n">
         <v>0.185</v>
@@ -3405,10 +3384,10 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="B51" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="C51" t="n">
         <v>1</v>
@@ -3423,10 +3402,10 @@
         <v>20</v>
       </c>
       <c r="G51" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H51" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I51" t="n">
         <v>0.17</v>
@@ -3446,7 +3425,7 @@
       <c r="N51"/>
       <c r="O51"/>
       <c r="P51" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="Q51" t="s">
         <v>23</v>
@@ -3454,10 +3433,10 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="B52" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="C52" t="n">
         <v>2</v>
@@ -3472,10 +3451,10 @@
         <v>20</v>
       </c>
       <c r="G52" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H52" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I52" t="n">
         <v>0.08</v>
@@ -3495,7 +3474,7 @@
       <c r="N52"/>
       <c r="O52"/>
       <c r="P52" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="Q52" t="s">
         <v>23</v>
@@ -3503,10 +3482,10 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="B53" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="C53" t="n">
         <v>3</v>
@@ -3521,10 +3500,10 @@
         <v>20</v>
       </c>
       <c r="G53" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H53" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I53" t="n">
         <v>0.185</v>
@@ -3544,7 +3523,7 @@
       <c r="N53"/>
       <c r="O53"/>
       <c r="P53" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="Q53" t="s">
         <v>23</v>
@@ -3552,10 +3531,10 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="B54" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="C54" t="n">
         <v>1</v>
@@ -3573,7 +3552,7 @@
         <v>45</v>
       </c>
       <c r="H54" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="I54" t="n">
         <v>0.215</v>
@@ -3593,10 +3572,10 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="B55" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="C55" t="n">
         <v>1</v>
@@ -3614,7 +3593,7 @@
         <v>45</v>
       </c>
       <c r="H55" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="I55" t="n">
         <v>0.18</v>
@@ -3644,10 +3623,10 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="B56" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="C56" t="n">
         <v>2</v>
@@ -3665,7 +3644,7 @@
         <v>45</v>
       </c>
       <c r="H56" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="I56" t="n">
         <v>0.115</v>
@@ -3695,10 +3674,10 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="B57" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="C57" t="n">
         <v>3</v>
@@ -3716,7 +3695,7 @@
         <v>45</v>
       </c>
       <c r="H57" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="I57" t="n">
         <v>0.12</v>
@@ -3746,10 +3725,10 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="B58" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="C58" t="n">
         <v>1</v>
@@ -3767,7 +3746,7 @@
         <v>45</v>
       </c>
       <c r="H58" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="I58" t="n">
         <v>0.25</v>
@@ -3797,10 +3776,10 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="B59" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="C59" t="n">
         <v>2</v>
@@ -3818,7 +3797,7 @@
         <v>45</v>
       </c>
       <c r="H59" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="I59" t="n">
         <v>0.225</v>
@@ -3848,10 +3827,10 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="B60" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="C60" t="n">
         <v>1</v>
@@ -3869,7 +3848,7 @@
         <v>45</v>
       </c>
       <c r="H60" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="I60" t="n">
         <v>0.105</v>
@@ -3899,10 +3878,10 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="B61" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="C61" t="n">
         <v>2</v>
@@ -3920,7 +3899,7 @@
         <v>45</v>
       </c>
       <c r="H61" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="I61" t="n">
         <v>0.215</v>
@@ -3950,10 +3929,10 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="B62" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="C62" t="n">
         <v>3</v>
@@ -3971,7 +3950,7 @@
         <v>45</v>
       </c>
       <c r="H62" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="I62" t="n">
         <v>0.125</v>
@@ -4001,10 +3980,10 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="B63" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="C63" t="n">
         <v>1</v>
@@ -4052,10 +4031,10 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="B64" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="C64" t="n">
         <v>2</v>
@@ -4103,10 +4082,10 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="B65" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="C65" t="n">
         <v>1</v>
@@ -4154,10 +4133,10 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="B66" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="C66" t="n">
         <v>2</v>
@@ -4205,10 +4184,10 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="B67" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="C67" t="n">
         <v>1</v>
@@ -4256,10 +4235,10 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="B68" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="C68" t="n">
         <v>1</v>
@@ -4274,10 +4253,10 @@
         <v>20</v>
       </c>
       <c r="G68" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H68" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I68" t="n">
         <v>0.055</v>
@@ -4295,7 +4274,7 @@
       <c r="N68"/>
       <c r="O68"/>
       <c r="P68" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="Q68" t="s">
         <v>23</v>
@@ -4303,10 +4282,10 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="B69" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="C69" t="n">
         <v>3</v>
@@ -4321,10 +4300,10 @@
         <v>20</v>
       </c>
       <c r="G69" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H69" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I69" t="n">
         <v>0.065</v>
@@ -4354,10 +4333,10 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="B70" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="C70" t="n">
         <v>4</v>
@@ -4372,10 +4351,10 @@
         <v>20</v>
       </c>
       <c r="G70" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H70" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I70" t="n">
         <v>0.145</v>
@@ -4405,10 +4384,10 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="B71" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="C71" t="n">
         <v>1</v>
@@ -4423,10 +4402,10 @@
         <v>20</v>
       </c>
       <c r="G71" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H71" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I71" t="n">
         <v>0.18</v>
@@ -4456,10 +4435,10 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="B72" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="C72" t="n">
         <v>2</v>
@@ -4474,10 +4453,10 @@
         <v>20</v>
       </c>
       <c r="G72" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H72" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I72" t="n">
         <v>0.195</v>
@@ -4507,10 +4486,10 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="B73" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="C73" t="n">
         <v>3</v>
@@ -4525,10 +4504,10 @@
         <v>20</v>
       </c>
       <c r="G73" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H73" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I73" t="n">
         <v>0.18</v>
@@ -4558,10 +4537,10 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="B74" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="C74" t="n">
         <v>1</v>
@@ -4576,10 +4555,10 @@
         <v>20</v>
       </c>
       <c r="G74" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H74" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I74" t="n">
         <v>0.09</v>
@@ -4609,10 +4588,10 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="B75" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="C75" t="n">
         <v>2</v>
@@ -4627,10 +4606,10 @@
         <v>20</v>
       </c>
       <c r="G75" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H75" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I75" t="n">
         <v>0.085</v>
@@ -4660,10 +4639,10 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="B76" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="C76" t="n">
         <v>3</v>
@@ -4678,10 +4657,10 @@
         <v>20</v>
       </c>
       <c r="G76" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H76" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I76" t="n">
         <v>0.035</v>
@@ -4696,7 +4675,7 @@
         <v>22.7272727272727</v>
       </c>
       <c r="M76" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="N76" t="n">
         <v>0.035</v>
@@ -4711,10 +4690,10 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="B77" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="C77" t="n">
         <v>1</v>
@@ -4729,10 +4708,10 @@
         <v>20</v>
       </c>
       <c r="G77" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H77" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I77" t="n">
         <v>0.075</v>
@@ -4747,7 +4726,7 @@
         <v>36.5853658536585</v>
       </c>
       <c r="M77" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="N77" t="n">
         <v>0.075</v>
@@ -4762,10 +4741,10 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="B78" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="C78" t="n">
         <v>2</v>
@@ -4780,10 +4759,10 @@
         <v>20</v>
       </c>
       <c r="G78" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H78" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I78" t="n">
         <v>0.16</v>
@@ -4798,7 +4777,7 @@
         <v>51.1182108626198</v>
       </c>
       <c r="M78" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="N78" t="n">
         <v>0.16</v>
@@ -4813,10 +4792,10 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="B79" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="C79" t="n">
         <v>1</v>
@@ -4831,10 +4810,10 @@
         <v>20</v>
       </c>
       <c r="G79" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H79" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I79" t="n">
         <v>0.065</v>
@@ -4864,10 +4843,10 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="B80" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="C80" t="n">
         <v>2</v>
@@ -4882,10 +4861,10 @@
         <v>20</v>
       </c>
       <c r="G80" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H80" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I80" t="n">
         <v>0.27</v>
@@ -4909,7 +4888,7 @@
         <v>0</v>
       </c>
       <c r="P80" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="Q80" t="s">
         <v>23</v>
@@ -4917,10 +4896,10 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="B81" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="C81" t="n">
         <v>1</v>
@@ -4956,7 +4935,7 @@
       <c r="N81"/>
       <c r="O81"/>
       <c r="P81" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="Q81" t="s">
         <v>23</v>
@@ -4964,10 +4943,10 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="B82" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="C82" t="n">
         <v>2</v>
@@ -5000,7 +4979,7 @@
         <v>36.144578313253</v>
       </c>
       <c r="M82" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="N82" t="n">
         <v>0.09</v>
@@ -5015,10 +4994,10 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="B83" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="C83" t="n">
         <v>3</v>
@@ -5066,10 +5045,10 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="B84" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="C84" t="n">
         <v>5</v>
@@ -5102,7 +5081,7 @@
         <v>74.7126436781609</v>
       </c>
       <c r="M84" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="N84" t="n">
         <v>0.26</v>
@@ -5117,10 +5096,10 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="B85" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="C85" t="n">
         <v>1</v>
@@ -5168,10 +5147,10 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="B86" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="C86" t="n">
         <v>2</v>
@@ -5219,10 +5198,10 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="B87" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="C87" t="n">
         <v>3</v>
@@ -5270,10 +5249,10 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="B88" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="C88" t="n">
         <v>1</v>
@@ -5315,7 +5294,7 @@
         <v>0</v>
       </c>
       <c r="P88" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="Q88" t="s">
         <v>23</v>
@@ -5323,10 +5302,10 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B89" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="C89" t="n">
         <v>3</v>
@@ -5374,10 +5353,10 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="B90" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="C90" t="n">
         <v>1</v>
@@ -5425,10 +5404,10 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="B91" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="C91" t="n">
         <v>2</v>
@@ -5464,7 +5443,7 @@
       <c r="N91"/>
       <c r="O91"/>
       <c r="P91" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="Q91" t="s">
         <v>23</v>
@@ -5472,10 +5451,10 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="B92" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="C92" t="n">
         <v>3</v>
@@ -5517,7 +5496,7 @@
         <v>0</v>
       </c>
       <c r="P92" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="Q92" t="s">
         <v>23</v>
@@ -5525,10 +5504,10 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="B93" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="C93" t="n">
         <v>4</v>
@@ -5576,10 +5555,10 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="B94" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="C94" t="n">
         <v>1</v>
@@ -5621,7 +5600,7 @@
         <v>0</v>
       </c>
       <c r="P94" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="Q94" t="s">
         <v>23</v>
@@ -5629,10 +5608,10 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="B95" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="C95" t="n">
         <v>2</v>
@@ -5680,10 +5659,10 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="B96" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="C96" t="n">
         <v>3</v>
@@ -5725,7 +5704,7 @@
         <v>0</v>
       </c>
       <c r="P96" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="Q96" t="s">
         <v>23</v>
@@ -5733,10 +5712,10 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="B97" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="C97" t="n">
         <v>1</v>
@@ -5784,10 +5763,10 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="B98" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="C98" t="n">
         <v>2</v>
@@ -5835,10 +5814,10 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="B99" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="C99" t="n">
         <v>1</v>
@@ -5886,10 +5865,10 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="B100" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="C100" t="n">
         <v>2</v>
@@ -5937,10 +5916,10 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="B101" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="C101" t="n">
         <v>2</v>
@@ -5988,10 +5967,10 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="B102" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="C102" t="n">
         <v>3</v>
@@ -6039,10 +6018,10 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="B103" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="C103" t="n">
         <v>4</v>
@@ -6090,10 +6069,10 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="B104" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="C104" t="n">
         <v>1</v>
@@ -6141,10 +6120,10 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="B105" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="C105" t="n">
         <v>3</v>

</xml_diff>